<commit_message>
round 3 report. almost done. some discrepnacies remain. the authors very likely forgot to update all of the outputs in the paper
</commit_message>
<xml_diff>
--- a/package-output-map.xlsx
+++ b/package-output-map.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diegogonzalezgonzalez/Desktop/Data Replicator/JPE/JPE-Soltas-20241011/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80955A17-F4B9-464C-A03B-E20461122A4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ACDBFFA-CB8E-354B-8DC4-621571FCC078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16100" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="227">
   <si>
     <t>Data Preparation Program</t>
   </si>
@@ -718,9 +718,6 @@
   </si>
   <si>
     <t>welfare_for_table_crrautil.dta</t>
-  </si>
-  <si>
-    <t>No</t>
   </si>
 </sst>
 </file>
@@ -1226,7 +1223,7 @@
         <v>98</v>
       </c>
       <c r="H4" t="s">
-        <v>227</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">

</xml_diff>